<commit_message>
Criação dos testes para UC - 03
</commit_message>
<xml_diff>
--- a/4.Teste/BRA - Roteiro de Teste.xlsx
+++ b/4.Teste/BRA - Roteiro de Teste.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fabioas\Development\bra-brasileirao_analyst\4.Teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1FB4B2-FCC9-478F-BACE-AE6F4D9A8A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D767A164-2A65-4FFE-8076-CFF707425B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="913" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="913" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Capa" sheetId="1" r:id="rId1"/>
     <sheet name="AUX" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet name="UCS001" sheetId="3" r:id="rId3"/>
     <sheet name="UCS002" sheetId="26" r:id="rId4"/>
+    <sheet name="UCS003" sheetId="27" r:id="rId5"/>
+    <sheet name="UCS004" sheetId="29" r:id="rId6"/>
+    <sheet name="UCS005" sheetId="28" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="___xlfn_IFERROR">NA()</definedName>
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="36">
   <si>
     <t>Caso de Uso</t>
   </si>
@@ -92,9 +95,6 @@
     <t>Pré-Condições:</t>
   </si>
   <si>
-    <t>O usuário deve estar logado no Sistema e possuir perfil de acesso à funcionalidade .</t>
-  </si>
-  <si>
     <t>Totais</t>
   </si>
   <si>
@@ -117,6 +117,43 @@
   </si>
   <si>
     <t>BRA - Brasileirão Analyst</t>
+  </si>
+  <si>
+    <t>UCS003</t>
+  </si>
+  <si>
+    <t>UCS004</t>
+  </si>
+  <si>
+    <t>UCS005</t>
+  </si>
+  <si>
+    <t>Extrair dados dos clubes e dos atletas</t>
+  </si>
+  <si>
+    <t>Execução da rotina agendada pelo serviço interno (Scheduler)</t>
+  </si>
+  <si>
+    <t>BRA - Massa de Testes UC03</t>
+  </si>
+  <si>
+    <t>Execução com sucesso da carga de dados via Scraper</t>
+  </si>
+  <si>
+    <t>Erro na execução de extração de dados</t>
+  </si>
+  <si>
+    <t>Disparo do serviço de extração</t>
+  </si>
+  <si>
+    <t>Dados atualizados dos 20
+clubes e seus respectivos atletas persistidos no banco de dados.</t>
+  </si>
+  <si>
+    <t>Disparo do serviço de extração sem conexão com a internet ou banco de dados</t>
+  </si>
+  <si>
+    <t>Sistema registra log de erro no terminal.</t>
   </si>
 </sst>
 </file>
@@ -409,7 +446,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -708,6 +745,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -726,7 +796,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -797,6 +867,12 @@
     <xf numFmtId="0" fontId="23" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -812,11 +888,29 @@
     <xf numFmtId="0" fontId="23" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="15">
@@ -1285,23 +1379,23 @@
     <row r="1" spans="2:12" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="18" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="24"/>
-      <c r="C2" s="37" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="37"/>
-      <c r="K2" s="37"/>
-      <c r="L2" s="38"/>
+      <c r="C2" s="32" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="33"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="25"/>
       <c r="G3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L3" s="26"/>
     </row>
@@ -1329,7 +1423,9 @@
       <c r="C5" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="22"/>
+      <c r="D5" s="22">
+        <v>4</v>
+      </c>
       <c r="F5" s="20"/>
       <c r="G5" s="20"/>
       <c r="H5" s="20"/>
@@ -1340,7 +1436,9 @@
       <c r="C6" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="22"/>
+      <c r="D6" s="22">
+        <v>3</v>
+      </c>
       <c r="F6" s="20"/>
       <c r="G6" s="20"/>
       <c r="H6" s="20"/>
@@ -1348,8 +1446,12 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="25"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="22"/>
+      <c r="C7" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="22">
+        <v>2</v>
+      </c>
       <c r="F7" s="20"/>
       <c r="G7" s="20"/>
       <c r="H7" s="20"/>
@@ -1357,8 +1459,12 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="25"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="22"/>
+      <c r="C8" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="22">
+        <v>4</v>
+      </c>
       <c r="F8" s="20"/>
       <c r="G8" s="20"/>
       <c r="H8" s="20"/>
@@ -1366,8 +1472,12 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="25"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="22"/>
+      <c r="C9" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="22">
+        <v>2</v>
+      </c>
       <c r="F9" s="20"/>
       <c r="G9" s="20"/>
       <c r="H9" s="20"/>
@@ -1466,7 +1576,7 @@
     <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="25"/>
       <c r="C20" s="23" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D20" s="23"/>
       <c r="F20" s="17"/>
@@ -1478,11 +1588,11 @@
       <c r="B21" s="25"/>
       <c r="C21" s="22">
         <f>COUNTA(C5:C19)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D21" s="22">
         <f>SUM(D5:D19)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F21" s="3">
         <f>SUM(F5:F19)</f>
@@ -1573,31 +1683,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
     </row>
     <row r="2" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="33">
-        <v>6</v>
-      </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
+      <c r="A2" s="35">
+        <v>0</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
     </row>
     <row r="3" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="36"/>
+      <c r="B4" s="38"/>
       <c r="C4" s="15"/>
     </row>
     <row r="5" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
@@ -1612,17 +1722,15 @@
         <v>15</v>
       </c>
       <c r="B6" s="8"/>
-      <c r="C6" s="16" t="s">
-        <v>16</v>
-      </c>
+      <c r="C6" s="16"/>
     </row>
     <row r="7" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="8" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>18</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>19</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>13</v>
@@ -1631,13 +1739,13 @@
         <v>14</v>
       </c>
       <c r="E8" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="31" t="s">
-        <v>21</v>
-      </c>
       <c r="G8" s="31" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1826,31 +1934,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
     </row>
     <row r="2" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A2" s="33">
-        <v>6</v>
-      </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
+      <c r="A2" s="35">
+        <v>0</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
     </row>
     <row r="3" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="36"/>
+      <c r="B4" s="38"/>
       <c r="C4" s="15"/>
     </row>
     <row r="5" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
@@ -1865,17 +1973,15 @@
         <v>15</v>
       </c>
       <c r="B6" s="8"/>
-      <c r="C6" s="16" t="s">
-        <v>16</v>
-      </c>
+      <c r="C6" s="16"/>
     </row>
     <row r="7" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="8" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>18</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>19</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>13</v>
@@ -1884,13 +1990,13 @@
         <v>14</v>
       </c>
       <c r="E8" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="31" t="s">
-        <v>21</v>
-      </c>
       <c r="G8" s="31" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2061,4 +2167,755 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Página &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71F60E2E-A501-4152-A762-911DC46BEE93}">
+  <dimension ref="A1:W19"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="62.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.44140625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="28.5546875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="38.6640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.109375" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+    </row>
+    <row r="2" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A2" s="35">
+        <v>2</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+    </row>
+    <row r="3" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+    </row>
+    <row r="4" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="38"/>
+      <c r="C4" s="15"/>
+    </row>
+    <row r="5" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="15"/>
+    </row>
+    <row r="6" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="16"/>
+    </row>
+    <row r="7" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="55.2" x14ac:dyDescent="0.25">
+      <c r="A9" s="44">
+        <v>1</v>
+      </c>
+      <c r="B9" s="45" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="45" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="39"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="5"/>
+    </row>
+    <row r="10" spans="1:23" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="A10" s="46">
+        <v>2</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="5"/>
+    </row>
+    <row r="11" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="40"/>
+      <c r="B11" s="41"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="42"/>
+    </row>
+    <row r="12" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="40"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+    </row>
+    <row r="13" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="40"/>
+      <c r="B13" s="41"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="43"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+    </row>
+    <row r="14" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="40"/>
+      <c r="B14" s="41"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="41"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="40"/>
+      <c r="B15" s="41"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="43"/>
+      <c r="F15" s="43"/>
+      <c r="G15" s="43"/>
+    </row>
+    <row r="16" spans="1:23" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="40"/>
+      <c r="B16" s="41"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="42"/>
+      <c r="G16" s="42"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="40"/>
+      <c r="B17" s="41"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="43"/>
+      <c r="G17" s="43"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="40"/>
+      <c r="B18" s="41"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="43"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="40"/>
+      <c r="B19" s="41"/>
+      <c r="C19" s="41"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="43"/>
+      <c r="G19" s="43"/>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:B4"/>
+  </mergeCells>
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0527777777777778" bottom="1.0527777777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <headerFooter alignWithMargins="0">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Página &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D072D88-11EC-4610-B00A-25B80911B562}">
+  <dimension ref="A1:W19"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.109375" style="4" customWidth="1"/>
+    <col min="3" max="3" width="32.44140625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="28.5546875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="38.6640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.109375" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+    </row>
+    <row r="2" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A2" s="35">
+        <v>0</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+    </row>
+    <row r="3" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+    </row>
+    <row r="4" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="38"/>
+      <c r="C4" s="15"/>
+    </row>
+    <row r="5" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="15"/>
+    </row>
+    <row r="6" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="8"/>
+      <c r="C6" s="16"/>
+    </row>
+    <row r="7" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10">
+        <v>1</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="5"/>
+    </row>
+    <row r="10" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9">
+        <v>2</v>
+      </c>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="5"/>
+    </row>
+    <row r="11" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="9">
+        <v>3</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+    </row>
+    <row r="12" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="9">
+        <v>4</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+    </row>
+    <row r="13" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="9">
+        <v>5</v>
+      </c>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+    </row>
+    <row r="14" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="10">
+        <v>6</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="9">
+        <v>7</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+    </row>
+    <row r="16" spans="1:23" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="9">
+        <v>8</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="9">
+        <v>9</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="9">
+        <v>10</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="10">
+        <v>11</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:B4"/>
+  </mergeCells>
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0527777777777778" bottom="1.0527777777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <headerFooter alignWithMargins="0">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Página &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84173073-7FBE-4C64-858D-7748D0584C8D}">
+  <dimension ref="A1:W19"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.109375" style="4" customWidth="1"/>
+    <col min="3" max="3" width="32.44140625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="28.5546875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="38.6640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="15.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.109375" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+    </row>
+    <row r="2" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A2" s="35">
+        <v>0</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+    </row>
+    <row r="3" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+    </row>
+    <row r="4" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="38"/>
+      <c r="C4" s="15"/>
+    </row>
+    <row r="5" spans="1:23" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="15"/>
+    </row>
+    <row r="6" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="8"/>
+      <c r="C6" s="16"/>
+    </row>
+    <row r="7" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10">
+        <v>1</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="5"/>
+    </row>
+    <row r="10" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9">
+        <v>2</v>
+      </c>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="5"/>
+    </row>
+    <row r="11" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="9">
+        <v>3</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+    </row>
+    <row r="12" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="9">
+        <v>4</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+    </row>
+    <row r="13" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="9">
+        <v>5</v>
+      </c>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+    </row>
+    <row r="14" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="10">
+        <v>6</v>
+      </c>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="9">
+        <v>7</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+    </row>
+    <row r="16" spans="1:23" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="9">
+        <v>8</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="9">
+        <v>9</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="9">
+        <v>10</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="10">
+        <v>11</v>
+      </c>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:B4"/>
+  </mergeCells>
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0527777777777778" bottom="1.0527777777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <headerFooter alignWithMargins="0">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Página &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>